<commit_message>
v.2.35 Staff Template Fix
</commit_message>
<xml_diff>
--- a/public/files/StaffTemplateNew.xlsx
+++ b/public/files/StaffTemplateNew.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30110"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7B6A67B7-E632-4FFE-9C89-4EFBBB67CA4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C15586E7-2406-4DBC-A4EF-AB15F3CCA144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,48 +34,45 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Designation</t>
   </si>
   <si>
-    <t>Resident</t>
+    <t>Resident *</t>
   </si>
   <si>
     <t>Location Access</t>
   </si>
   <si>
-    <t>IC No.</t>
-  </si>
-  <si>
-    <t>Passport No.</t>
+    <t>IC No. / Passport *</t>
   </si>
   <si>
     <t>Visa Expiry</t>
   </si>
   <si>
-    <t>Date of Birth</t>
-  </si>
-  <si>
-    <t>Gender</t>
-  </si>
-  <si>
-    <t>Full Name</t>
+    <t>Date of Birth *</t>
+  </si>
+  <si>
+    <t>Gender *</t>
+  </si>
+  <si>
+    <t>Full Name *</t>
   </si>
   <si>
     <t>Name on Staff Pass</t>
   </si>
   <si>
-    <t>Staff No.</t>
-  </si>
-  <si>
-    <t>Contact No.</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Department</t>
+    <t>Staff No. *</t>
+  </si>
+  <si>
+    <t>Contact No. *</t>
+  </si>
+  <si>
+    <t>Email *</t>
+  </si>
+  <si>
+    <t>Department *</t>
   </si>
   <si>
     <t>Address</t>
@@ -93,13 +90,13 @@
     <t>Postcode</t>
   </si>
   <si>
-    <t>License Class</t>
-  </si>
-  <si>
-    <t>License Expiry</t>
-  </si>
-  <si>
-    <t>Status</t>
+    <t>License Class *</t>
+  </si>
+  <si>
+    <t>License Expiry *</t>
+  </si>
+  <si>
+    <t>Status *</t>
   </si>
 </sst>
 </file>
@@ -123,7 +120,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -159,14 +156,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -485,96 +505,108 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="5.42578125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="4.140625" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2"/>
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="V1" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="D1:E1"/>
+  </mergeCells>
+  <dataValidations count="3">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error=" You must fill out this field" sqref="B1" xr:uid="{0CF7E419-3675-4BEF-B7F0-333381729EA8}">
+      <formula1>LEN(A2)&gt;0</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="You must fill out this field" sqref="D1 U1 G1 H1 I1 K1 L1 M1 N1 T1" xr:uid="{EE9D1DEC-7D98-4840-82C2-3656E45AAEB3}">
+      <formula1>LEN(A2)&gt;0</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="You must fill out this field " sqref="V1" xr:uid="{90F5CD0F-2919-46AE-AACF-DE803D859C5A}">
+      <formula1>LEN(A2)&gt;0</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Migration + Staff Template Amendments
</commit_message>
<xml_diff>
--- a/public/files/StaffTemplateNew.xlsx
+++ b/public/files/StaffTemplateNew.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C15586E7-2406-4DBC-A4EF-AB15F3CCA144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\conra\Desktop\Byte_ Projects\VMS 2.0\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8F4E914-5D9B-4E0D-9A68-8870BDFC9E94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -15,17 +20,6 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>
     </ext>
@@ -34,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Designation</t>
   </si>
@@ -72,9 +66,6 @@
     <t>Email *</t>
   </si>
   <si>
-    <t>Department *</t>
-  </si>
-  <si>
     <t>Address</t>
   </si>
   <si>
@@ -90,20 +81,20 @@
     <t>Postcode</t>
   </si>
   <si>
-    <t>License Class *</t>
-  </si>
-  <si>
-    <t>License Expiry *</t>
-  </si>
-  <si>
-    <t>Status *</t>
+    <t xml:space="preserve">Department </t>
+  </si>
+  <si>
+    <t xml:space="preserve">License Class </t>
+  </si>
+  <si>
+    <t xml:space="preserve">License Expiry </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -178,13 +169,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -501,111 +492,105 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1796875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.1796875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="13" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="5.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="5.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="4.1796875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2"/>
-      <c r="F1" s="3" t="s">
+      <c r="E1" s="4"/>
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="T1" s="3" t="s">
+      <c r="T1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="U1" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="V1" s="3" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D1:E1"/>
   </mergeCells>
-  <dataValidations count="3">
+  <dataValidations count="2">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error=" You must fill out this field" sqref="B1" xr:uid="{0CF7E419-3675-4BEF-B7F0-333381729EA8}">
       <formula1>LEN(A2)&gt;0</formula1>
     </dataValidation>
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="You must fill out this field" sqref="D1 U1 G1 H1 I1 K1 L1 M1 N1 T1" xr:uid="{EE9D1DEC-7D98-4840-82C2-3656E45AAEB3}">
       <formula1>LEN(A2)&gt;0</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="You must fill out this field " sqref="V1" xr:uid="{90F5CD0F-2919-46AE-AACF-DE803D859C5A}">
-      <formula1>LEN(A2)&gt;0</formula1>
-    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>